<commit_message>
fix: touch backend to ensure reload
</commit_message>
<xml_diff>
--- a/backend/data/correlation_analysis.xlsx
+++ b/backend/data/correlation_analysis.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:V22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,104 +436,114 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>귀하의 연령은?</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>귀하의 학력은?</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>귀하의 직업은? (복수로 체크 가능)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>귀하의 월소득 수준은?</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>귀하가 거주하는 지역은 ?</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>귀하의 종교는 ?</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>귀하의 성경 통독 횟수는 ?</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>귀하의 교회 직분은 무엇입니까?</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>성별</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>연령</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>학력</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>월평균소득</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>재직기간</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>직위</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>전문분야</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>고용형태</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>se1</t>
-        </is>
-      </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>se2</t>
+          <t>독11</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>se3</t>
+          <t>독12</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>직무만족</t>
+          <t>독13</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>정서적몰입</t>
+          <t>종1</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>자기효능감</t>
+          <t>매11</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>새 1</t>
+          <t>매12</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>새 2</t>
+          <t>매13</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>새 3</t>
+          <t>매2</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>새 4</t>
+          <t>조11</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>새 5</t>
+          <t>조12</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>조13</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>조14</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>성별</t>
+          <t>귀하의 연령은?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -559,16 +569,18 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>연령</t>
+          <t>귀하의 학력은?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>.029</t>
+          <t>.152**</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -593,21 +605,23 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>학력</t>
+          <t>귀하의 직업은? (복수로 체크 가능)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>.045</t>
+          <t>-.021</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>.242***</t>
+          <t>-.199***</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -631,26 +645,28 @@
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>월평균소득</t>
+          <t>귀하의 월소득 수준은?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-.104</t>
+          <t>.180***</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>.217***</t>
+          <t>.298***</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>.056</t>
+          <t>-.394***</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -673,31 +689,33 @@
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>재직기간</t>
+          <t>귀하가 거주하는 지역은 ?</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>-.081</t>
+          <t>-.116*</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>.719***</t>
+          <t>.014</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>.227***</t>
+          <t>-.065</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>.358***</t>
+          <t>.045</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -719,36 +737,38 @@
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>직위</t>
+          <t>귀하의 종교는 ?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>.046</t>
+          <t>-.142**</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-.396***</t>
+          <t>-.162**</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-.298***</t>
+          <t>.149**</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-.188**</t>
+          <t>-.139**</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>-.388***</t>
+          <t>-.016</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -769,41 +789,43 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>전문분야</t>
+          <t>귀하의 성경 통독 횟수는 ?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>.071</t>
+          <t>.334***</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-.067</t>
+          <t>.166***</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>.082</t>
+          <t>.015</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-.124*</t>
+          <t>.151**</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>-.087</t>
+          <t>.041</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>.110</t>
+          <t>-.234***</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -823,46 +845,48 @@
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>고용형태</t>
+          <t>귀하의 교회 직분은 무엇입니까?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>.208***</t>
+          <t>.336***</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>-.047</t>
+          <t>.232***</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>.088</t>
+          <t>.047</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-.264***</t>
+          <t>.053</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>-.150*</t>
+          <t>-.088</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>.200***</t>
+          <t>.097*</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>.174**</t>
+          <t>.210***</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -881,51 +905,53 @@
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>se1</t>
+          <t>성별</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>.097</t>
+          <t>.321***</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>.064</t>
+          <t>.191***</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>.197***</t>
+          <t>-.074</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>.018</t>
+          <t>.110*</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>.113</t>
+          <t>.002</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>-.207***</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>.080</t>
+          <t>.332***</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>.013</t>
+          <t>.113*</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -943,56 +969,58 @@
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>se2</t>
+          <t>독11</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>-.049</t>
+          <t>.046</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>.050</t>
+          <t>-.038</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>.199***</t>
+          <t>.004</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>.114</t>
+          <t>.042</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>.068</t>
+          <t>-.073</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-.047</t>
+          <t>.107*</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>-.070</t>
+          <t>.073</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>-.115*</t>
+          <t>.063</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>.524***</t>
+          <t>.031</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1009,61 +1037,63 @@
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>se3</t>
+          <t>독12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>-.044</t>
+          <t>-.033</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>.088</t>
+          <t>-.134**</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>.138*</t>
+          <t>.063</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>.120*</t>
+          <t>-.060</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>.167**</t>
+          <t>-.055</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-.080</t>
+          <t>.098*</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>.011</t>
+          <t>-.054</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>-.080</t>
+          <t>-.057</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>.527***</t>
+          <t>-.102*</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>.504***</t>
+          <t>.672***</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1079,66 +1109,68 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>직무만족</t>
+          <t>독13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>.015</t>
+          <t>-.018</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>.075</t>
+          <t>-.064</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>.213***</t>
+          <t>.021</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>.044</t>
+          <t>.060</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>.149*</t>
+          <t>-.081</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-.082</t>
+          <t>.014</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>.046</t>
+          <t>-.038</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>-.027</t>
+          <t>-.087</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>.486***</t>
+          <t>.003</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>.533***</t>
+          <t>.578***</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>.590***</t>
+          <t>.635***</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1153,71 +1185,73 @@
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>정서적몰입</t>
+          <t>종1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>.010</t>
+          <t>.026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>.166**</t>
+          <t>-.011</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>.176**</t>
+          <t>.065</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>.103</t>
+          <t>.034</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>.182**</t>
+          <t>-.066</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-.091</t>
+          <t>.084</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>-.024</t>
+          <t>.055</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>-.115*</t>
+          <t>-.003</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>.401***</t>
+          <t>-.023</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>.629***</t>
+          <t>.466***</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>.393***</t>
+          <t>.476***</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>.614***</t>
+          <t>.556***</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1231,76 +1265,78 @@
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>자기효능감</t>
+          <t>매11</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-.079</t>
+          <t>.022</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-.038</t>
+          <t>-.074</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>.126*</t>
+          <t>-.008</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>.131*</t>
+          <t>.037</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>.079</t>
+          <t>-.094</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>.002</t>
+          <t>.067</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>-.014</t>
+          <t>.027</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>-.092</t>
+          <t>-.062</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>.461***</t>
+          <t>-.003</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>.547***</t>
+          <t>.681***</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>.646***</t>
+          <t>.685***</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>.669***</t>
+          <t>.742***</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>.502***</t>
+          <t>.573***</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1313,81 +1349,83 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>새 1</t>
+          <t>매12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>-.001</t>
+          <t>-.019</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>.101</t>
+          <t>-.113*</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>.239***</t>
+          <t>.046</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>.081</t>
+          <t>-.024</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>.150*</t>
+          <t>-.005</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>-.049</t>
+          <t>.065</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>-.040</t>
+          <t>.042</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>-.005</t>
+          <t>-.029</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>.506***</t>
+          <t>-.072</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>.583***</t>
+          <t>.617***</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>.519***</t>
+          <t>.605***</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>.606***</t>
+          <t>.499***</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>.618***</t>
+          <t>.516***</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>.614***</t>
+          <t>.705***</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1399,86 +1437,88 @@
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>새 2</t>
+          <t>매13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>.027</t>
+          <t>-.022</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>.182**</t>
+          <t>-.079</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>.265***</t>
+          <t>.026</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>.123*</t>
+          <t>-.021</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>.121*</t>
+          <t>-.046</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>-.058</t>
+          <t>.081</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>.026</t>
+          <t>.041</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>.008</t>
+          <t>-.045</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>.370***</t>
+          <t>-.064</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>.489***</t>
+          <t>.573***</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>.520***</t>
+          <t>.538***</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>.539***</t>
+          <t>.509***</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>.589***</t>
+          <t>.590***</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>.520***</t>
+          <t>.612***</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>.658***</t>
+          <t>.675***</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1489,91 +1529,93 @@
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>새 3</t>
+          <t>매2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>.022</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>-.029</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>.015</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>.043</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>-.026</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>.044</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>.199***</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>.087</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>.102</t>
-        </is>
-      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-.035</t>
+          <t>.102*</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>.004</t>
+          <t>.078</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>-.049</t>
+          <t>-.043</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>.566***</t>
+          <t>-.003</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>.550***</t>
+          <t>.590***</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>.660***</t>
+          <t>.561***</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>.649***</t>
+          <t>.604***</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>.491***</t>
+          <t>.695***</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>.684***</t>
+          <t>.668***</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>.644***</t>
+          <t>.636***</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>.613***</t>
+          <t>.752***</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1583,96 +1625,98 @@
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>새 4</t>
+          <t>조11</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>-.001</t>
+          <t>-.048</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-.059</t>
+          <t>-.080</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>.006</t>
+          <t>.061</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>.032</t>
+          <t>-.023</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>-.043</t>
+          <t>.000</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>.032</t>
+          <t>.141**</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>.076</t>
+          <t>.090</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-.112</t>
+          <t>-.078</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>.052</t>
+          <t>-.026</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>.161**</t>
+          <t>.584***</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>.024</t>
+          <t>.559***</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-.043</t>
+          <t>.539***</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>.207***</t>
+          <t>.691***</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-.015</t>
+          <t>.643***</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-.051</t>
+          <t>.647***</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>.123*</t>
+          <t>.716***</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>.031</t>
+          <t>.802***</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -1681,104 +1725,328 @@
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>새 5</t>
+          <t>조12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>-.012</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>-.095</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>.088</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>-.035</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-.092</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>.021</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>-.003</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>-.083</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>-.055</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>.179**</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>.056</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>.013</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>.000</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>.054</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>-.077</t>
-        </is>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>.407***</t>
+          <t>-.018</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>.461***</t>
+          <t>.375***</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
+          <t>.376***</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>.388***</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>.499***</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>.465***</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>.496***</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>.515***</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>.572***</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>.594***</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>조13</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>-.067</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>-.104*</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>.074</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>-.091</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>-.010</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>.031</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>-.028</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>-.068</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>-.121*</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>.296***</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
           <t>.360***</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>.405***</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>.428***</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>.455***</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>.500***</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>.394***</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>.444***</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>.147*</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>.302***</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>.401***</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>.324***</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>.411***</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>.469***</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>.482***</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>.502***</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>.710***</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>조14</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>.004</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>-.053</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>.028</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>-.011</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-.004</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>.059</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>.068</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>-.089</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>.021</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>.438***</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>.414***</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>.409***</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>.700***</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>.492***</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>.506***</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>.628***</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>.684***</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>.694***</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>.653***</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>.659***</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>